<commit_message>
feat: graphy 26년2Q 데이터 업데이트 및 분석결과 추가, kyungnam task_list 수정
</commit_message>
<xml_diff>
--- a/graphy/task_list_graphy.xlsx
+++ b/graphy/task_list_graphy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\lbh00\OneDrive\문서\감사\감사자료\audit-automation\graphy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6528E7EC-478C-45E1-94AE-7943D442D286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1EC10C-319F-4349-8AA9-934C4F29868B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -24,12 +24,25 @@
     <sheet name="host1_외상매출매입상계" sheetId="9" r:id="rId9"/>
     <sheet name="host2_분개장AI분석" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="84">
   <si>
     <t>작업명</t>
   </si>
@@ -251,13 +264,52 @@
   </si>
   <si>
     <t>월별트렌드분석</t>
+  </si>
+  <si>
+    <t>기준월</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>당좌예금</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>보통예금</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>외화예금</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>기타제예금</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>정기예.적금</t>
+  </si>
+  <si>
+    <t>이자수익</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>보험료</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>대변만</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>차변만</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -300,6 +352,13 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -336,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -357,6 +416,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1092,7 +1152,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.9140625" style="6" customWidth="1"/>
@@ -1172,16 +1232,13 @@
         <v>47</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>42</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>8</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
@@ -1189,16 +1246,13 @@
         <v>47</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>8</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
@@ -1206,16 +1260,13 @@
         <v>47</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>8</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
@@ -1223,24 +1274,21 @@
         <v>47</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>8</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>53</v>
+        <v>47</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>79</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>42</v>
@@ -1251,13 +1299,13 @@
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>54</v>
+        <v>47</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>80</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>8</v>
@@ -1265,13 +1313,13 @@
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>55</v>
+        <v>47</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>81</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>8</v>
@@ -1279,10 +1327,10 @@
     </row>
     <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>56</v>
+        <v>47</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>42</v>
@@ -1290,35 +1338,145 @@
       <c r="F12" s="6" t="s">
         <v>8</v>
       </c>
+      <c r="G12" s="6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>57</v>
+        <v>47</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>49</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>8</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B21" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1331,44 +1489,45 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.4140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.25" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.4140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.6640625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1381,80 +1540,81 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="17" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="17" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" customWidth="1"/>
-    <col min="2" max="2" width="63.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="63.83203125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" style="8" customWidth="1"/>
+    <col min="4" max="16384" width="8.6640625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="D2" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="D3" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="D4" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="8" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1571,91 +1731,121 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="17" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="11.08203125" customWidth="1"/>
+    <col min="2" max="2" width="12.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>61</v>
       </c>
       <c r="B1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>28</v>
       </c>
       <c r="B2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>30</v>
       </c>
       <c r="B3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>31</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>32</v>
       </c>
       <c r="B5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>33</v>
       </c>
       <c r="B6" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>34</v>
       </c>
       <c r="B7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>35</v>
       </c>
       <c r="B8" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>36</v>
       </c>
       <c r="B9" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>37</v>
       </c>
       <c r="B10" t="s">
         <v>41</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>